<commit_message>
Updated mobile call functions
</commit_message>
<xml_diff>
--- a/data/user_variables.xlsx
+++ b/data/user_variables.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03EA205F-A9D2-44CF-8904-734924AB5E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11355" windowHeight="6525"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserVariablesGOLIAT" sheetId="1" r:id="rId1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="87">
   <si>
     <t>Variable name</t>
   </si>
@@ -129,9 +130,6 @@
     <t>Mobile calling, far-field exposure</t>
   </si>
   <si>
-    <t>Mobile data transfer</t>
-  </si>
-  <si>
     <t>Laptop use</t>
   </si>
   <si>
@@ -168,15 +166,9 @@
     <t>implemented</t>
   </si>
   <si>
-    <t>Proportion of time mobile phone is held against ear during mobile call. For now, we assume the remaining time the phone is 50% in speaker mode and 50% with headphones, but we can change this in the future.</t>
-  </si>
-  <si>
     <t>not implemented</t>
   </si>
   <si>
-    <t>Proportion of time headphones are used during mobile call when mobile phone is NOT held against ear</t>
-  </si>
-  <si>
     <t>Proportion of time phone is in pocket vs in front of face vs away during phone call with headphone</t>
   </si>
   <si>
@@ -244,12 +236,60 @@
   </si>
   <si>
     <t>home: yes, work: no</t>
+  </si>
+  <si>
+    <t>mpc_headp_prop</t>
+  </si>
+  <si>
+    <t>hotspot_duration</t>
+  </si>
+  <si>
+    <t>smartwatch_duration</t>
+  </si>
+  <si>
+    <t>tracker_duration</t>
+  </si>
+  <si>
+    <t>vr_duration</t>
+  </si>
+  <si>
+    <t>headphone_duration</t>
+  </si>
+  <si>
+    <t>smarthome_duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile data </t>
+  </si>
+  <si>
+    <t>Mobile data</t>
+  </si>
+  <si>
+    <t>implement?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proportion of time mobile phone is held against ear during mobile call. </t>
+  </si>
+  <si>
+    <t>Proportion of time headphones are used during mobile call when mobile phone is NOT held against ear. We assume that the remaining proportion of time, the phone is used in speaker mode.</t>
+  </si>
+  <si>
+    <t>Not in GOLIAT?</t>
+  </si>
+  <si>
+    <t>Not in GOLIAT</t>
+  </si>
+  <si>
+    <t>Could be derived from GOLIAT questionnaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Don't have this info in GOLIAT </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -265,7 +305,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -286,19 +326,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -315,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -329,7 +375,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -337,6 +383,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -618,22 +667,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" style="2" customWidth="1"/>
-    <col min="2" max="3" width="20.85546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="50.42578125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="19.26953125" style="2" customWidth="1"/>
+    <col min="2" max="3" width="20.81640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="19.26953125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="50.453125" style="2" customWidth="1"/>
     <col min="7" max="7" width="22" style="2" customWidth="1"/>
-    <col min="8" max="8" width="24.28515625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="60.85546875" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="2"/>
+    <col min="8" max="8" width="24.26953125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="60.81640625" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -641,7 +690,7 @@
         <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -662,205 +711,205 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>4</v>
+    <row r="2" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>71</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>47</v>
+      <c r="C2" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D2" s="2">
-        <v>425</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>47</v>
+      <c r="C3" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D3" s="2">
-        <v>0.66</v>
+        <v>425</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.66</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="5" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C5" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="B6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="2">
         <v>10800</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" s="2" t="s">
+      <c r="F6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="2">
+      <c r="B7" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="2">
         <v>0.5</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="2">
-        <v>204</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>31</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>47</v>
+      <c r="C8" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D8" s="2">
+        <v>204</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="2">
         <v>0.9</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="B10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="2">
         <v>4371</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1617</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>6</v>
@@ -869,18 +918,18 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>47</v>
+        <v>37</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D11" s="2">
-        <v>59400</v>
+        <v>1617</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>6</v>
@@ -889,234 +938,274 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>39</v>
+      </c>
       <c r="B12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="2">
+        <v>59400</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="2">
+        <v>8280</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B19" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C19" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="2">
+      <c r="I20" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D21" s="2">
         <v>0.5</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B13" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B22" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B24" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B25" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="2">
-        <v>0</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="2">
-        <v>0</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D22" s="2">
-        <v>0</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D23" s="2">
-        <v>0</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D24" s="2">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D25" s="2">
-        <v>8280</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>64</v>
+      <c r="I25" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:I1" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I25">
+      <sortCondition ref="C1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed typo in readme
</commit_message>
<xml_diff>
--- a/data/user_variables.xlsx
+++ b/data/user_variables.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03EA205F-A9D2-44CF-8904-734924AB5E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6DD8DD-758B-4E5A-8978-46410686C292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-12345" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserVariablesGOLIAT" sheetId="1" r:id="rId1"/>

</xml_diff>